<commit_message>
now with teaching evals
</commit_message>
<xml_diff>
--- a/assets/evaluationkit-questionmapper.xlsx
+++ b/assets/evaluationkit-questionmapper.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davisjam/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davisjam/Downloads/purdue-tenure-packet-generator/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA554ABA-B4A3-EE49-A9FC-602BEE87B5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D741CFB8-5A22-054F-8541-37DAE7945BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1900" yWindow="1820" windowWidth="27240" windowHeight="16440" xr2:uid="{37535F24-3F79-6942-A99C-C04D16879D1F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="66">
   <si>
     <t>QuestionKey</t>
   </si>
@@ -186,6 +186,57 @@
   </si>
   <si>
     <t>737250-0</t>
+  </si>
+  <si>
+    <t>614817-0</t>
+  </si>
+  <si>
+    <t>614818-0</t>
+  </si>
+  <si>
+    <t>614819-0</t>
+  </si>
+  <si>
+    <t>614821-0</t>
+  </si>
+  <si>
+    <t>614822-0</t>
+  </si>
+  <si>
+    <t>614823-0</t>
+  </si>
+  <si>
+    <t>614824-0</t>
+  </si>
+  <si>
+    <t>614825-0</t>
+  </si>
+  <si>
+    <t>614826-0</t>
+  </si>
+  <si>
+    <t>679118-0</t>
+  </si>
+  <si>
+    <t>679119-0</t>
+  </si>
+  <si>
+    <t>679120-0</t>
+  </si>
+  <si>
+    <t>679121-0</t>
+  </si>
+  <si>
+    <t>679122-0</t>
+  </si>
+  <si>
+    <t>679123-0</t>
+  </si>
+  <si>
+    <t>679124-0</t>
+  </si>
+  <si>
+    <t>679125-0</t>
   </si>
 </sst>
 </file>
@@ -557,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B82D641-E984-B745-ADC1-52E6950AAF79}">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -868,6 +919,193 @@
         <v>36</v>
       </c>
     </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>62</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>64</v>
+      </c>
+      <c r="B44" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>65</v>
+      </c>
+      <c r="B45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>